<commit_message>
v3.5.1 - Backup 50 archivos, Excel con tipos animales y facturación
</commit_message>
<xml_diff>
--- a/upload/PLANTILLA_IMPORTACION_DATOS.xlsx
+++ b/upload/PLANTILLA_IMPORTACION_DATOS.xlsx
@@ -22,6 +22,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROMANEOS_HISTORICOS" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DESPACHOS_HISTORICOS" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FACTURAS_HISTORICAS" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRODUCTOS_VENDIBLES" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRECIOS_CLIENTE" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DETALLE_FACTURAS" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +34,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,8 +80,17 @@
       <i val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -109,6 +121,12 @@
         <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -136,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -159,6 +177,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -948,7 +970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -982,7 +1004,13 @@
           <t>Registre todas las tropas del año. Estado: DESPACHADO, FAENADO, etc. Fecha formato: DD/MM/AAAA</t>
         </is>
       </c>
-    </row>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tipos de animales: TO:5, VA:3, NO:2 (formato: TIPO:CANTIDAD, separados por coma)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -1019,47 +1047,52 @@
           <t>cantidadCabezas</t>
         </is>
       </c>
-      <c r="H4" s="12" t="inlineStr">
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>tiposAnimales</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
         <is>
           <t>dte</t>
         </is>
       </c>
-      <c r="I4" s="12" t="inlineStr">
+      <c r="J4" s="12" t="inlineStr">
         <is>
           <t>guia</t>
         </is>
       </c>
-      <c r="J4" s="12" t="inlineStr">
+      <c r="K4" s="12" t="inlineStr">
         <is>
           <t>corralNombre</t>
         </is>
       </c>
-      <c r="K4" s="12" t="inlineStr">
+      <c r="L4" s="12" t="inlineStr">
         <is>
           <t>pesoBruto</t>
         </is>
       </c>
-      <c r="L4" s="12" t="inlineStr">
+      <c r="M4" s="12" t="inlineStr">
         <is>
           <t>pesoTara</t>
         </is>
       </c>
-      <c r="M4" s="12" t="inlineStr">
+      <c r="N4" s="12" t="inlineStr">
         <is>
           <t>pesoNeto</t>
         </is>
       </c>
-      <c r="N4" s="12" t="inlineStr">
+      <c r="O4" s="12" t="inlineStr">
         <is>
           <t>fechaRecepcion</t>
         </is>
       </c>
-      <c r="O4" s="12" t="inlineStr">
+      <c r="P4" s="12" t="inlineStr">
         <is>
           <t>estado</t>
         </is>
       </c>
-      <c r="P4" s="12" t="inlineStr">
+      <c r="Q4" s="12" t="inlineStr">
         <is>
           <t>observaciones</t>
         </is>
@@ -1101,21 +1134,16 @@
           <t>OBLIGATORIO</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>OBLIGATORIO</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>OBLIGATORIO</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>OPCIONAL</t>
-        </is>
-      </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
           <t>OPCIONAL</t>
@@ -1131,17 +1159,22 @@
           <t>OPCIONAL</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>OPCIONAL</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="inlineStr">
         <is>
           <t>OBLIGATORIO</t>
         </is>
       </c>
-      <c r="O5" s="7" t="inlineStr">
+      <c r="P5" s="7" t="inlineStr">
         <is>
           <t>OBLIGATORIO</t>
         </is>
       </c>
-      <c r="P5" s="8" t="inlineStr">
+      <c r="Q5" s="8" t="inlineStr">
         <is>
           <t>OPCIONAL</t>
         </is>
@@ -1183,47 +1216,47 @@
           <t>25</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>DTE-123456</t>
         </is>
       </c>
-      <c r="I6" s="9" t="inlineStr">
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>GUIA-789012</t>
         </is>
       </c>
-      <c r="J6" s="9" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>Corral 1</t>
         </is>
       </c>
-      <c r="K6" s="9" t="inlineStr">
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>15000</t>
         </is>
       </c>
-      <c r="L6" s="9" t="inlineStr">
+      <c r="M6" s="9" t="inlineStr">
         <is>
           <t>5000</t>
         </is>
       </c>
-      <c r="M6" s="9" t="inlineStr">
+      <c r="N6" s="9" t="inlineStr">
         <is>
           <t>10000</t>
         </is>
       </c>
-      <c r="N6" s="9" t="inlineStr">
+      <c r="O6" s="9" t="inlineStr">
         <is>
           <t>02/01/2026</t>
         </is>
       </c>
-      <c r="O6" s="9" t="inlineStr">
+      <c r="P6" s="9" t="inlineStr">
         <is>
           <t>DESPACHADO</t>
         </is>
       </c>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="Q6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1253,47 +1286,47 @@
           <t>15</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="I7" s="9" t="inlineStr">
         <is>
           <t>DTE-234567</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr">
+      <c r="J7" s="9" t="inlineStr">
         <is>
           <t>GUIA-890123</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="K7" s="9" t="inlineStr">
         <is>
           <t>Corral 2</t>
         </is>
       </c>
-      <c r="K7" s="9" t="inlineStr">
+      <c r="L7" s="9" t="inlineStr">
         <is>
           <t>9000</t>
         </is>
       </c>
-      <c r="L7" s="9" t="inlineStr">
+      <c r="M7" s="9" t="inlineStr">
         <is>
           <t>3000</t>
         </is>
       </c>
-      <c r="M7" s="9" t="inlineStr">
+      <c r="N7" s="9" t="inlineStr">
         <is>
           <t>6000</t>
         </is>
       </c>
-      <c r="N7" s="9" t="inlineStr">
+      <c r="O7" s="9" t="inlineStr">
         <is>
           <t>03/01/2026</t>
         </is>
       </c>
-      <c r="O7" s="9" t="inlineStr">
+      <c r="P7" s="9" t="inlineStr">
         <is>
           <t>DESPACHADO</t>
         </is>
       </c>
-      <c r="P7" s="9" t="inlineStr">
+      <c r="Q7" s="9" t="inlineStr">
         <is>
           <t>Tropa pequeña</t>
         </is>
@@ -1331,47 +1364,47 @@
           <t>30</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr">
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t>DTE-345678</t>
         </is>
       </c>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="J8" s="9" t="inlineStr">
         <is>
           <t>GUIA-901234</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="K8" s="9" t="inlineStr">
         <is>
           <t>Corral 1</t>
         </is>
       </c>
-      <c r="K8" s="9" t="inlineStr">
+      <c r="L8" s="9" t="inlineStr">
         <is>
           <t>18000</t>
         </is>
       </c>
-      <c r="L8" s="9" t="inlineStr">
+      <c r="M8" s="9" t="inlineStr">
         <is>
           <t>6000</t>
         </is>
       </c>
-      <c r="M8" s="9" t="inlineStr">
+      <c r="N8" s="9" t="inlineStr">
         <is>
           <t>12000</t>
         </is>
       </c>
-      <c r="N8" s="9" t="inlineStr">
+      <c r="O8" s="9" t="inlineStr">
         <is>
           <t>04/01/2026</t>
         </is>
       </c>
-      <c r="O8" s="9" t="inlineStr">
+      <c r="P8" s="9" t="inlineStr">
         <is>
           <t>DESPACHADO</t>
         </is>
       </c>
-      <c r="P8" s="9" t="inlineStr"/>
+      <c r="Q8" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1672,7 +1705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1700,7 +1733,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Registro de pesajes. Denticion: 0, 2, 4, 6, 8 dientes. Rinde se calcula automáticamente si no lo tiene.</t>
+          <t>Registro de pesajes. Denticion: 0, 2, 4, 6, 8 dientes. Rinde se calcula automáticamente si no lo tiene. PrecioKg: precio por kg para facturación.</t>
         </is>
       </c>
     </row>
@@ -1768,6 +1801,11 @@
       <c r="M4" s="12" t="inlineStr">
         <is>
           <t>observaciones</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>precioKg</t>
         </is>
       </c>
     </row>
@@ -2839,6 +2877,553 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>PRODUCTOS VENDIBLES (Catálogo para Facturación)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Productos y servicios facturables. Categorías: PRODUCTO_CARNICO, SERVICIO_FAENA, OTROS. Alícuota IVA: 10.5 o 21.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>codigo</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>descripcion</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>unidadMedida</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>precioBase</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>alicuotaIva</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>esActivo</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MR001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MEDIA RES BOVINA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Media res de bovino completa</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PRODUCTO_CARNICO</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CD001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CUARTO DELANTERO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Cuarto delantero de bovino</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PRODUCTO_CARNICO</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CT001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CUARTO TRASERO</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Cuarto trasero de bovino</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PRODUCTO_CARNICO</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SF001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SERVICIO FAENA BOVINO</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Servicio de faena bovina por animal</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SERVICIO_FAENA</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G8" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Incluye todo el proceso</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SF002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SERVICIO FAENA EQUINO</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Servicio de faena equina por animal</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SERVICIO_FAENA</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>18000</v>
+      </c>
+      <c r="G9" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MN001</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MENUDENCIAS VARIAS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Menudencias de bovino</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PRODUCTO_CARNICO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G10" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CR001</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CUERO BOVINO</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Cuero de bovino</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>OTROS</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>PRECIOS ESPECIALES POR CLIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Precios especiales acordados con clientes. Anular fechaHasta para precio vigente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>clienteCUIT</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>productoCodigo</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>precioEspecial</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>fechaDesde</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>fechaHasta</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>observaciones</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>DETALLE DE FACTURAS (Items facturados)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Detalle de cada item en las facturas. TipoProducto: MEDIA_RES, CUARTO_DELANTERO, CUARTO_TRASERO, MENUDENCIA, OTRO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>facturaNumero</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>productoCodigo</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>tipoProducto</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>descripcion</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>cantidad</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>precioUnitario</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>subtotal</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>tropaCodigo</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>garron</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>pesoKg</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>observaciones</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
v3.6.4 - Sistema FIFO completo, API PDF trazabilidad, mejoras en control de vencimientos
</commit_message>
<xml_diff>
--- a/upload/PLANTILLA_IMPORTACION_DATOS.xlsx
+++ b/upload/PLANTILLA_IMPORTACION_DATOS.xlsx
@@ -22,9 +22,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROMANEOS_HISTORICOS" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DESPACHOS_HISTORICOS" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FACTURAS_HISTORICAS" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRODUCTOS_VENDIBLES" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRECIOS_CLIENTE" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DETALLE_FACTURAS" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,17 +77,8 @@
       <i val="1"/>
       <sz val="9"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -121,12 +109,6 @@
         <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -154,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -177,10 +159,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -970,7 +948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1004,13 +982,7 @@
           <t>Registre todas las tropas del año. Estado: DESPACHADO, FAENADO, etc. Fecha formato: DD/MM/AAAA</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Tipos de animales: TO:5, VA:3, NO:2 (formato: TIPO:CANTIDAD, separados por coma)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+    </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -1047,52 +1019,47 @@
           <t>cantidadCabezas</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>tiposAnimales</t>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>dte</t>
         </is>
       </c>
       <c r="I4" s="12" t="inlineStr">
         <is>
-          <t>dte</t>
+          <t>guia</t>
         </is>
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>guia</t>
+          <t>corralNombre</t>
         </is>
       </c>
       <c r="K4" s="12" t="inlineStr">
         <is>
-          <t>corralNombre</t>
+          <t>pesoBruto</t>
         </is>
       </c>
       <c r="L4" s="12" t="inlineStr">
         <is>
-          <t>pesoBruto</t>
+          <t>pesoTara</t>
         </is>
       </c>
       <c r="M4" s="12" t="inlineStr">
         <is>
-          <t>pesoTara</t>
+          <t>pesoNeto</t>
         </is>
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>pesoNeto</t>
+          <t>fechaRecepcion</t>
         </is>
       </c>
       <c r="O4" s="12" t="inlineStr">
         <is>
-          <t>fechaRecepcion</t>
+          <t>estado</t>
         </is>
       </c>
       <c r="P4" s="12" t="inlineStr">
-        <is>
-          <t>estado</t>
-        </is>
-      </c>
-      <c r="Q4" s="12" t="inlineStr">
         <is>
           <t>observaciones</t>
         </is>
@@ -1134,47 +1101,47 @@
           <t>OBLIGATORIO</t>
         </is>
       </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>OBLIGATORIO</t>
+        </is>
+      </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
           <t>OBLIGATORIO</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>OPCIONAL</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>OPCIONAL</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>OPCIONAL</t>
+        </is>
+      </c>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>OPCIONAL</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
         <is>
           <t>OBLIGATORIO</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
-        <is>
-          <t>OPCIONAL</t>
-        </is>
-      </c>
-      <c r="L5" s="8" t="inlineStr">
-        <is>
-          <t>OPCIONAL</t>
-        </is>
-      </c>
-      <c r="M5" s="8" t="inlineStr">
-        <is>
-          <t>OPCIONAL</t>
-        </is>
-      </c>
-      <c r="N5" s="8" t="inlineStr">
-        <is>
-          <t>OPCIONAL</t>
-        </is>
-      </c>
       <c r="O5" s="7" t="inlineStr">
         <is>
           <t>OBLIGATORIO</t>
         </is>
       </c>
-      <c r="P5" s="7" t="inlineStr">
-        <is>
-          <t>OBLIGATORIO</t>
-        </is>
-      </c>
-      <c r="Q5" s="8" t="inlineStr">
+      <c r="P5" s="8" t="inlineStr">
         <is>
           <t>OPCIONAL</t>
         </is>
@@ -1216,47 +1183,47 @@
           <t>25</t>
         </is>
       </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>DTE-123456</t>
+        </is>
+      </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>DTE-123456</t>
+          <t>GUIA-789012</t>
         </is>
       </c>
       <c r="J6" s="9" t="inlineStr">
         <is>
-          <t>GUIA-789012</t>
+          <t>Corral 1</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
         <is>
-          <t>Corral 1</t>
+          <t>15000</t>
         </is>
       </c>
       <c r="L6" s="9" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>02/01/2026</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr">
         <is>
-          <t>02/01/2026</t>
-        </is>
-      </c>
-      <c r="P6" s="9" t="inlineStr">
-        <is>
           <t>DESPACHADO</t>
         </is>
       </c>
-      <c r="Q6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1286,47 +1253,47 @@
           <t>15</t>
         </is>
       </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>DTE-234567</t>
+        </is>
+      </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>DTE-234567</t>
+          <t>GUIA-890123</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
-          <t>GUIA-890123</t>
+          <t>Corral 2</t>
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr">
         <is>
-          <t>Corral 2</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>9000</t>
+          <t>3000</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>6000</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>6000</t>
+          <t>03/01/2026</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr">
         <is>
-          <t>03/01/2026</t>
+          <t>DESPACHADO</t>
         </is>
       </c>
       <c r="P7" s="9" t="inlineStr">
-        <is>
-          <t>DESPACHADO</t>
-        </is>
-      </c>
-      <c r="Q7" s="9" t="inlineStr">
         <is>
           <t>Tropa pequeña</t>
         </is>
@@ -1364,47 +1331,47 @@
           <t>30</t>
         </is>
       </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>DTE-345678</t>
+        </is>
+      </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>DTE-345678</t>
+          <t>GUIA-901234</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr">
         <is>
-          <t>GUIA-901234</t>
+          <t>Corral 1</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>Corral 1</t>
+          <t>18000</t>
         </is>
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>18000</t>
+          <t>6000</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>6000</t>
+          <t>12000</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>12000</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr">
         <is>
-          <t>04/01/2026</t>
-        </is>
-      </c>
-      <c r="P8" s="9" t="inlineStr">
-        <is>
           <t>DESPACHADO</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr"/>
+      <c r="P8" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1705,7 +1672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1733,7 +1700,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Registro de pesajes. Denticion: 0, 2, 4, 6, 8 dientes. Rinde se calcula automáticamente si no lo tiene. PrecioKg: precio por kg para facturación.</t>
+          <t>Registro de pesajes. Denticion: 0, 2, 4, 6, 8 dientes. Rinde se calcula automáticamente si no lo tiene.</t>
         </is>
       </c>
     </row>
@@ -1801,11 +1768,6 @@
       <c r="M4" s="12" t="inlineStr">
         <is>
           <t>observaciones</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>precioKg</t>
         </is>
       </c>
     </row>
@@ -2877,553 +2839,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="13" t="inlineStr">
-        <is>
-          <t>PRODUCTOS VENDIBLES (Catálogo para Facturación)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Productos y servicios facturables. Categorías: PRODUCTO_CARNICO, SERVICIO_FAENA, OTROS. Alícuota IVA: 10.5 o 21.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>codigo</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>nombre</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>descripcion</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>categoria</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>unidadMedida</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>precioBase</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>alicuotaIva</t>
-        </is>
-      </c>
-      <c r="H4" s="14" t="inlineStr">
-        <is>
-          <t>esActivo</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>observaciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>MR001</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>MEDIA RES BOVINA</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Media res de bovino completa</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>PRODUCTO_CARNICO</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="G5" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CD001</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>CUARTO DELANTERO</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Cuarto delantero de bovino</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>PRODUCTO_CARNICO</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>3200</v>
-      </c>
-      <c r="G6" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CT001</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>CUARTO TRASERO</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Cuarto trasero de bovino</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>PRODUCTO_CARNICO</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>3800</v>
-      </c>
-      <c r="G7" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>SF001</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>SERVICIO FAENA BOVINO</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Servicio de faena bovina por animal</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>SERVICIO_FAENA</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>UN</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>15000</v>
-      </c>
-      <c r="G8" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Incluye todo el proceso</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>SF002</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>SERVICIO FAENA EQUINO</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Servicio de faena equina por animal</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>SERVICIO_FAENA</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>UN</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G9" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MN001</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>MENUDENCIAS VARIAS</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Menudencias de bovino</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>PRODUCTO_CARNICO</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G10" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CR001</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>CUERO BOVINO</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Cuero de bovino</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>OTROS</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>UN</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G11" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="13" t="inlineStr">
-        <is>
-          <t>PRECIOS ESPECIALES POR CLIENTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Precios especiales acordados con clientes. Anular fechaHasta para precio vigente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>clienteCUIT</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>productoCodigo</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>precioEspecial</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>fechaDesde</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>fechaHasta</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>observaciones</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="13" t="inlineStr">
-        <is>
-          <t>DETALLE DE FACTURAS (Items facturados)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Detalle de cada item en las facturas. TipoProducto: MEDIA_RES, CUARTO_DELANTERO, CUARTO_TRASERO, MENUDENCIA, OTRO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>facturaNumero</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>productoCodigo</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>tipoProducto</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>descripcion</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>cantidad</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>unidad</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>precioUnitario</t>
-        </is>
-      </c>
-      <c r="H4" s="14" t="inlineStr">
-        <is>
-          <t>subtotal</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>tropaCodigo</t>
-        </is>
-      </c>
-      <c r="J4" s="14" t="inlineStr">
-        <is>
-          <t>garron</t>
-        </is>
-      </c>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>pesoKg</t>
-        </is>
-      </c>
-      <c r="L4" s="14" t="inlineStr">
-        <is>
-          <t>observaciones</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>